<commit_message>
v2 excellence pass for all 20 AI agent kits
Add 04-examples, 06-scorecard, 07-artifacts, VERSION and CHANGELOG per kit.
Excellence generator, Marketing Excel Example Acme Week tab, docs.

Co-authored-by: RevenueSystemsEngineer <samuelfreemanjobs-hash@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ai-agent-team/products/agent-03-marketing-planner-agent-kit/03-templates/Marketing-Command-Center.xlsx
+++ b/ai-agent-team/products/agent-03-marketing-planner-agent-kit/03-templates/Marketing-Command-Center.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Content Calendar" sheetId="4" r:id="rId4"/>
     <sheet name="Campaigns" sheetId="5" r:id="rId5"/>
     <sheet name="Lead Sources" sheetId="6" r:id="rId6"/>
+    <sheet name="Example Acme Week" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -1964,4 +1965,132 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D9"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Example only — Acme Digital Studio (delete or replace)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Metric</v>
+      </c>
+      <c r="B2" t="str">
+        <v>This Week</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Last Week</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Goal</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Website sessions</v>
+      </c>
+      <c r="B3">
+        <v>420</v>
+      </c>
+      <c r="C3">
+        <v>380</v>
+      </c>
+      <c r="D3">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Email subscribers</v>
+      </c>
+      <c r="B4">
+        <v>28</v>
+      </c>
+      <c r="C4">
+        <v>24</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Leads</v>
+      </c>
+      <c r="B5">
+        <v>9</v>
+      </c>
+      <c r="C5">
+        <v>7</v>
+      </c>
+      <c r="D5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Sales calls booked</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Revenue ($)</v>
+      </c>
+      <c r="B7">
+        <v>1240</v>
+      </c>
+      <c r="C7">
+        <v>980</v>
+      </c>
+      <c r="D7">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Email open rate %</v>
+      </c>
+      <c r="B8">
+        <v>38</v>
+      </c>
+      <c r="C8">
+        <v>35</v>
+      </c>
+      <c r="D8">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Social saves</v>
+      </c>
+      <c r="B9">
+        <v>64</v>
+      </c>
+      <c r="C9">
+        <v>51</v>
+      </c>
+      <c r="D9">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>